<commit_message>
2026-08-02 sweep: fresh fetch validating the FX fix and standardized insider data
Live test of both changes from the previous commit. New snapshot, coverage
report, and _MarketCache confirm: foreign-currency cash/crypto now
correctly convert to SEK (previously silent zeros), and Handelsbanken/
Investor insider transactions came back real and populated in the
standardized equities[ticker]["insider_activity_se"] field. Reasoning
agents (valuation, macro-regime, portfolio, thesis-review) are running
against this data next; council report to follow in a separate commit.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WjQXsnKMoHNoBeicmtVwVc
</commit_message>
<xml_diff>
--- a/master.xlsx
+++ b/master.xlsx
@@ -624,7 +624,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-08-02 09:52 UTC</t>
+          <t>2026-08-02 10:03 UTC</t>
         </is>
       </c>
     </row>
@@ -801,7 +801,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-08-02T09:51:47.510979+00:00</t>
+          <t>2026-08-02T10:03:21.567440+00:00</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -834,7 +834,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-08-02T09:51:47.510979+00:00</t>
+          <t>2026-08-02T10:03:21.567440+00:00</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -862,7 +862,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-08-02T09:51:47.510979+00:00</t>
+          <t>2026-08-02T10:03:21.567440+00:00</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -922,7 +922,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-08-02T09:51:47.510979+00:00</t>
+          <t>2026-08-02T10:03:21.567440+00:00</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -980,7 +980,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1620.75</v>
+        <v>1620.59</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -989,11 +989,11 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-08-02T09:51:47.510979+00:00</t>
+          <t>2026-08-02T10:03:21.567440+00:00</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>17898.2664</v>
+        <v>17896.4995</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -1022,7 +1022,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-08-02T09:51:47.510979+00:00</t>
+          <t>2026-08-02T10:03:21.567440+00:00</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-08-02T09:51:47.510979+00:00</t>
+          <t>2026-08-02T10:03:21.567440+00:00</t>
         </is>
       </c>
       <c r="E12" t="n">

</xml_diff>

<commit_message>
First sweep under the consolidated report format (2026-08-02)
Full pipeline test after today's FX-fix and insider-standardization work:
journal -> prep -> valuation/macro-regime/portfolio/thesis-review -> council
-> journal. Report at reports/2026-08-02-sweep.md; Notes-sheet row logged
for next sweep's reconciliation. Controller's first live run under the new
5-persona structure to follow in a separate commit.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WjQXsnKMoHNoBeicmtVwVc
</commit_message>
<xml_diff>
--- a/master.xlsx
+++ b/master.xlsx
@@ -4955,7 +4955,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5702,6 +5702,28 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>sweep-2026-08-02</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>First sweep under consolidated single-report format (reports/2026-08-02-sweep.md), nothing to reconcile against. Headline items: (1) Two Pending Orders awaiting execution confirmation - Visa 7,500 SEK and Schneider Electric (SU.PA) 5,000 SEK, both committed 2026-07-29. (2) Settings sheet contribution_routing_default still says 100% to Secure tier, conflicts with current Medium-tier priority given 90.1%-vs-60% Secure drift - needs update. (3) Open decision: whether to write SHB-A.ST/INVE-A.ST theses now on insider-buying signal (Boman/Lundberg SHB-A.ST, Cederholm INVE-A.ST) vs wait for confirmed fundamentals (INVE-A.ST CIK fetch broken, SHB-A.ST PE is manual override); both at/near 52w highs, no written thesis exists. (4) Open decision: Swedbank AF fund cost basis unknown - request from Swedbank statement vs leave as legacy holding.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>